<commit_message>
feat: implementar extração de dados do IBGE e processamento de parquets
- Adicionada integração com a API de agregados do IBGE para estimativa populacional.
- Implementada lógica de conversão de dados da API para DataFrame com indexação por 'Ano'.
- Criada função genérica  para exportação em Excel (.xlsx).
- Implementada função  para carregamento otimizado (colunas seletivas) e concatenação de múltiplos arquivos do SINAN.
- Adicionado tratamento de exceções para caminhos de diretórios e arquivos inexistentes.
</commit_message>
<xml_diff>
--- a/dados_filtrados/SINAN/estupros_viols_df.xlsx
+++ b/dados_filtrados/SINAN/estupros_viols_df.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="PwbAwu0YW2vY4QH04moKZsCBjDJxPbskCWIuAVZK9h8="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="3dWT0CerbOPAJSCGmC1SReak7bTwM3KPYxO2RXlLFN0="/>
     </ext>
   </extLst>
 </workbook>
@@ -558,10 +558,10 @@
         <v>25.17</v>
       </c>
       <c r="R2" s="2">
-        <v>1200.0</v>
+        <v>504.0</v>
       </c>
       <c r="S2" s="2">
-        <v>42.07</v>
+        <v>17.67</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
@@ -617,10 +617,10 @@
         <v>18.8</v>
       </c>
       <c r="R3" s="2">
-        <v>890.0</v>
+        <v>485.0</v>
       </c>
       <c r="S3" s="2">
-        <v>30.53</v>
+        <v>16.64</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
@@ -676,10 +676,10 @@
         <v>29.46</v>
       </c>
       <c r="R4" s="2">
-        <v>1266.0</v>
+        <v>731.0</v>
       </c>
       <c r="S4" s="2">
-        <v>42.52</v>
+        <v>24.55</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
@@ -735,10 +735,10 @@
         <v>50.14</v>
       </c>
       <c r="R5" s="2">
-        <v>2270.0</v>
+        <v>1240.0</v>
       </c>
       <c r="S5" s="2">
-        <v>74.68</v>
+        <v>40.8</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
@@ -794,10 +794,10 @@
         <v>66.12</v>
       </c>
       <c r="R6" s="2">
-        <v>2902.0</v>
+        <v>1477.0</v>
       </c>
       <c r="S6" s="2">
-        <v>97.56</v>
+        <v>49.65</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
@@ -853,10 +853,10 @@
         <v>82.48</v>
       </c>
       <c r="R7" s="2">
-        <v>3700.0</v>
+        <v>1768.0</v>
       </c>
       <c r="S7" s="2">
-        <v>122.71</v>
+        <v>58.63</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
@@ -912,10 +912,10 @@
         <v>83.5</v>
       </c>
       <c r="R8" s="2">
-        <v>3516.0</v>
+        <v>1530.0</v>
       </c>
       <c r="S8" s="2">
-        <v>115.08</v>
+        <v>50.08</v>
       </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
@@ -971,10 +971,10 @@
         <v>98.15</v>
       </c>
       <c r="R9" s="2">
-        <v>4123.0</v>
+        <v>1667.0</v>
       </c>
       <c r="S9" s="2">
-        <v>133.24</v>
+        <v>53.87</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
@@ -1030,10 +1030,10 @@
         <v>150.5</v>
       </c>
       <c r="R10" s="2">
-        <v>5938.0</v>
+        <v>2252.0</v>
       </c>
       <c r="S10" s="2">
-        <v>199.07</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
@@ -1089,10 +1089,10 @@
         <v>245.49</v>
       </c>
       <c r="R11" s="2">
-        <v>9522.0</v>
+        <v>2572.0</v>
       </c>
       <c r="S11" s="2">
-        <v>317.73</v>
+        <v>85.82</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>